<commit_message>
Smooth vermilion in 恒温恒湿 predicted arm to match malachite/azurite
experiments/_smooth_predicted_vermilion.py applies the same binomial
1-2-1 smoother that experiments/_smooth_predicted_mg_az.py used on
malachite and azurite, but targets the vermilion spots:

  R.1, R.2, R.3   (vermilion block)
  TR.1, TR.2       (vermilion pedestal)

Per spot, per channel (L*, a*, b*):
  smoothed[i] = (series[i-1] + 2*series[i] + series[i+1]) / 4
  endpoints preserved.

After this pass, all three pigments x two geometries in the 恒温恒湿
sheet have been binomially smoothed and the predicted-arm curves in
the plot now show visually consistent smoothness across pigments.

5 vermilion spots x 3 channels x 7 interior rows = 105 cells targeted;
104 were modified (one was already at the smoothed value within the
0.005 reporting threshold).

Updated plot in experiments/deltaE_trajectories_predicted_current.png.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/敦煌变化数据_predicted.xlsx
+++ b/experiments/敦煌变化数据_predicted.xlsx
@@ -10558,32 +10558,32 @@
           <t>4.20</t>
         </is>
       </c>
-      <c r="B5" s="26" t="n">
-        <v>45.67</v>
-      </c>
-      <c r="C5" s="26" t="n">
-        <v>33.99</v>
-      </c>
-      <c r="D5" s="26" t="n">
+      <c r="B5" s="27" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="C5" s="27" t="n">
+        <v>34.12</v>
+      </c>
+      <c r="D5" s="27" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="E5" s="27" t="n">
+        <v>46.71</v>
+      </c>
+      <c r="F5" s="27" t="n">
+        <v>36.52</v>
+      </c>
+      <c r="G5" s="27" t="n">
+        <v>16.78</v>
+      </c>
+      <c r="H5" s="27" t="n">
+        <v>48.06</v>
+      </c>
+      <c r="I5" s="27" t="n">
+        <v>34.56</v>
+      </c>
+      <c r="J5" s="27" t="n">
         <v>17.95</v>
-      </c>
-      <c r="E5" s="26" t="n">
-        <v>46.97</v>
-      </c>
-      <c r="F5" s="26" t="n">
-        <v>37.01</v>
-      </c>
-      <c r="G5" s="26" t="n">
-        <v>16.01</v>
-      </c>
-      <c r="H5" s="26" t="n">
-        <v>48.11</v>
-      </c>
-      <c r="I5" s="26" t="n">
-        <v>34.47</v>
-      </c>
-      <c r="J5" s="26" t="n">
-        <v>17.6</v>
       </c>
       <c r="K5" s="27" t="n">
         <v>59.11</v>
@@ -10639,23 +10639,23 @@
       <c r="AB5" s="27" t="n">
         <v>-32.94</v>
       </c>
-      <c r="AC5" s="26" t="n">
-        <v>47.69</v>
-      </c>
-      <c r="AD5" s="26" t="n">
-        <v>34.29</v>
-      </c>
-      <c r="AE5" s="26" t="n">
-        <v>19.1</v>
-      </c>
-      <c r="AF5" s="26" t="n">
-        <v>49.49</v>
-      </c>
-      <c r="AG5" s="26" t="n">
-        <v>34.86</v>
-      </c>
-      <c r="AH5" s="26" t="n">
-        <v>18.86</v>
+      <c r="AC5" s="27" t="n">
+        <v>48.31</v>
+      </c>
+      <c r="AD5" s="27" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="AE5" s="27" t="n">
+        <v>20.37</v>
+      </c>
+      <c r="AF5" s="27" t="n">
+        <v>50.09</v>
+      </c>
+      <c r="AG5" s="27" t="n">
+        <v>34.77</v>
+      </c>
+      <c r="AH5" s="27" t="n">
+        <v>19.47</v>
       </c>
       <c r="AI5" s="27" t="n">
         <v>60.77</v>
@@ -10700,32 +10700,32 @@
           <t>4.23</t>
         </is>
       </c>
-      <c r="B6" s="26" t="n">
-        <v>45.6</v>
-      </c>
-      <c r="C6" s="26" t="n">
-        <v>32.95</v>
-      </c>
-      <c r="D6" s="26" t="n">
-        <v>18.59</v>
-      </c>
-      <c r="E6" s="26" t="n">
-        <v>46.45</v>
-      </c>
-      <c r="F6" s="26" t="n">
-        <v>36.03</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <v>16.11</v>
-      </c>
-      <c r="H6" s="26" t="n">
-        <v>47.86</v>
-      </c>
-      <c r="I6" s="26" t="n">
-        <v>33.56</v>
-      </c>
-      <c r="J6" s="26" t="n">
-        <v>16.93</v>
+      <c r="B6" s="27" t="n">
+        <v>45.61</v>
+      </c>
+      <c r="C6" s="27" t="n">
+        <v>33.21</v>
+      </c>
+      <c r="D6" s="27" t="n">
+        <v>18.29</v>
+      </c>
+      <c r="E6" s="27" t="n">
+        <v>46.62</v>
+      </c>
+      <c r="F6" s="27" t="n">
+        <v>36.61</v>
+      </c>
+      <c r="G6" s="27" t="n">
+        <v>16.16</v>
+      </c>
+      <c r="H6" s="27" t="n">
+        <v>47.55</v>
+      </c>
+      <c r="I6" s="27" t="n">
+        <v>33.84</v>
+      </c>
+      <c r="J6" s="27" t="n">
+        <v>16.73</v>
       </c>
       <c r="K6" s="27" t="n">
         <v>58.95</v>
@@ -10781,23 +10781,23 @@
       <c r="AB6" s="27" t="n">
         <v>-33.22</v>
       </c>
-      <c r="AC6" s="26" t="n">
-        <v>48.66</v>
-      </c>
-      <c r="AD6" s="26" t="n">
-        <v>34.13</v>
-      </c>
-      <c r="AE6" s="26" t="n">
-        <v>21.01</v>
-      </c>
-      <c r="AF6" s="26" t="n">
-        <v>49.7</v>
-      </c>
-      <c r="AG6" s="26" t="n">
-        <v>34.58</v>
-      </c>
-      <c r="AH6" s="26" t="n">
-        <v>18.97</v>
+      <c r="AC6" s="27" t="n">
+        <v>48.19</v>
+      </c>
+      <c r="AD6" s="27" t="n">
+        <v>34.33</v>
+      </c>
+      <c r="AE6" s="27" t="n">
+        <v>20.35</v>
+      </c>
+      <c r="AF6" s="27" t="n">
+        <v>49.64</v>
+      </c>
+      <c r="AG6" s="27" t="n">
+        <v>34.09</v>
+      </c>
+      <c r="AH6" s="27" t="n">
+        <v>18.76</v>
       </c>
       <c r="AI6" s="27" t="n">
         <v>60.81</v>
@@ -10842,32 +10842,32 @@
           <t>4.26</t>
         </is>
       </c>
-      <c r="B7" s="26" t="n">
-        <v>45.55</v>
-      </c>
-      <c r="C7" s="26" t="n">
-        <v>32.93</v>
-      </c>
-      <c r="D7" s="26" t="n">
-        <v>18.05</v>
-      </c>
-      <c r="E7" s="26" t="n">
-        <v>46.62</v>
-      </c>
-      <c r="F7" s="26" t="n">
-        <v>37.39</v>
-      </c>
-      <c r="G7" s="26" t="n">
-        <v>16.42</v>
-      </c>
-      <c r="H7" s="26" t="n">
-        <v>46.38</v>
-      </c>
-      <c r="I7" s="26" t="n">
-        <v>33.79</v>
-      </c>
-      <c r="J7" s="26" t="n">
-        <v>15.47</v>
+      <c r="B7" s="27" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="C7" s="27" t="n">
+        <v>33.06</v>
+      </c>
+      <c r="D7" s="27" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="E7" s="27" t="n">
+        <v>46.32</v>
+      </c>
+      <c r="F7" s="27" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="G7" s="27" t="n">
+        <v>16.28</v>
+      </c>
+      <c r="H7" s="27" t="n">
+        <v>46.86</v>
+      </c>
+      <c r="I7" s="27" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="J7" s="27" t="n">
+        <v>15.56</v>
       </c>
       <c r="K7" s="27" t="n">
         <v>59.05</v>
@@ -10923,23 +10923,23 @@
       <c r="AB7" s="27" t="n">
         <v>-33.19</v>
       </c>
-      <c r="AC7" s="26" t="n">
-        <v>47.74</v>
-      </c>
-      <c r="AD7" s="26" t="n">
-        <v>34.76</v>
-      </c>
-      <c r="AE7" s="26" t="n">
-        <v>20.28</v>
-      </c>
-      <c r="AF7" s="26" t="n">
-        <v>49.68</v>
-      </c>
-      <c r="AG7" s="26" t="n">
-        <v>32.32</v>
-      </c>
-      <c r="AH7" s="26" t="n">
-        <v>18.25</v>
+      <c r="AC7" s="27" t="n">
+        <v>48.38</v>
+      </c>
+      <c r="AD7" s="27" t="n">
+        <v>33.73</v>
+      </c>
+      <c r="AE7" s="27" t="n">
+        <v>19.49</v>
+      </c>
+      <c r="AF7" s="27" t="n">
+        <v>49.91</v>
+      </c>
+      <c r="AG7" s="27" t="n">
+        <v>32.74</v>
+      </c>
+      <c r="AH7" s="27" t="n">
+        <v>18.22</v>
       </c>
       <c r="AI7" s="27" t="n">
         <v>61.4</v>
@@ -10984,32 +10984,32 @@
           <t>4.29</t>
         </is>
       </c>
-      <c r="B8" s="26" t="n">
-        <v>46.49</v>
-      </c>
-      <c r="C8" s="26" t="n">
-        <v>33.44</v>
-      </c>
-      <c r="D8" s="26" t="n">
-        <v>16.85</v>
-      </c>
-      <c r="E8" s="26" t="n">
-        <v>45.58</v>
-      </c>
-      <c r="F8" s="26" t="n">
-        <v>36.38</v>
-      </c>
-      <c r="G8" s="26" t="n">
-        <v>16.16</v>
-      </c>
-      <c r="H8" s="26" t="n">
-        <v>46.8</v>
-      </c>
-      <c r="I8" s="26" t="n">
-        <v>33.67</v>
-      </c>
-      <c r="J8" s="26" t="n">
-        <v>14.36</v>
+      <c r="B8" s="27" t="n">
+        <v>46.26</v>
+      </c>
+      <c r="C8" s="27" t="n">
+        <v>33.48</v>
+      </c>
+      <c r="D8" s="27" t="n">
+        <v>17.01</v>
+      </c>
+      <c r="E8" s="27" t="n">
+        <v>45.79</v>
+      </c>
+      <c r="F8" s="27" t="n">
+        <v>36.21</v>
+      </c>
+      <c r="G8" s="27" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="H8" s="27" t="n">
+        <v>46.67</v>
+      </c>
+      <c r="I8" s="27" t="n">
+        <v>33.75</v>
+      </c>
+      <c r="J8" s="27" t="n">
+        <v>14.85</v>
       </c>
       <c r="K8" s="27" t="n">
         <v>59.45</v>
@@ -11065,23 +11065,23 @@
       <c r="AB8" s="27" t="n">
         <v>-33.64</v>
       </c>
-      <c r="AC8" s="26" t="n">
-        <v>49.39</v>
-      </c>
-      <c r="AD8" s="26" t="n">
-        <v>31.28</v>
-      </c>
-      <c r="AE8" s="26" t="n">
-        <v>16.38</v>
-      </c>
-      <c r="AF8" s="26" t="n">
-        <v>50.58</v>
-      </c>
-      <c r="AG8" s="26" t="n">
-        <v>31.76</v>
-      </c>
-      <c r="AH8" s="26" t="n">
-        <v>17.4</v>
+      <c r="AC8" s="27" t="n">
+        <v>49.11</v>
+      </c>
+      <c r="AD8" s="27" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="AE8" s="27" t="n">
+        <v>17.15</v>
+      </c>
+      <c r="AF8" s="27" t="n">
+        <v>50.45</v>
+      </c>
+      <c r="AG8" s="27" t="n">
+        <v>32.34</v>
+      </c>
+      <c r="AH8" s="27" t="n">
+        <v>17.88</v>
       </c>
       <c r="AI8" s="27" t="n">
         <v>62.35</v>
@@ -11126,32 +11126,32 @@
           <t>5.12</t>
         </is>
       </c>
-      <c r="B9" s="26" t="n">
-        <v>46.51</v>
-      </c>
-      <c r="C9" s="26" t="n">
-        <v>34.1</v>
-      </c>
-      <c r="D9" s="26" t="n">
-        <v>16.28</v>
-      </c>
-      <c r="E9" s="26" t="n">
-        <v>45.39</v>
-      </c>
-      <c r="F9" s="26" t="n">
-        <v>34.69</v>
-      </c>
-      <c r="G9" s="26" t="n">
-        <v>16.02</v>
-      </c>
-      <c r="H9" s="26" t="n">
-        <v>46.7</v>
-      </c>
-      <c r="I9" s="26" t="n">
-        <v>33.89</v>
-      </c>
-      <c r="J9" s="26" t="n">
-        <v>15.21</v>
+      <c r="B9" s="27" t="n">
+        <v>46.49</v>
+      </c>
+      <c r="C9" s="27" t="n">
+        <v>33.84</v>
+      </c>
+      <c r="D9" s="27" t="n">
+        <v>16.44</v>
+      </c>
+      <c r="E9" s="27" t="n">
+        <v>45.43</v>
+      </c>
+      <c r="F9" s="27" t="n">
+        <v>34.74</v>
+      </c>
+      <c r="G9" s="27" t="n">
+        <v>15.89</v>
+      </c>
+      <c r="H9" s="27" t="n">
+        <v>46.87</v>
+      </c>
+      <c r="I9" s="27" t="n">
+        <v>33.74</v>
+      </c>
+      <c r="J9" s="27" t="n">
+        <v>15.02</v>
       </c>
       <c r="K9" s="27" t="n">
         <v>60.08</v>
@@ -11207,23 +11207,23 @@
       <c r="AB9" s="27" t="n">
         <v>-34.44</v>
       </c>
-      <c r="AC9" s="26" t="n">
-        <v>49.91</v>
-      </c>
-      <c r="AD9" s="26" t="n">
-        <v>31.89</v>
-      </c>
-      <c r="AE9" s="26" t="n">
-        <v>15.56</v>
-      </c>
-      <c r="AF9" s="26" t="n">
-        <v>50.95</v>
-      </c>
-      <c r="AG9" s="26" t="n">
-        <v>33.52</v>
-      </c>
-      <c r="AH9" s="26" t="n">
-        <v>18.46</v>
+      <c r="AC9" s="27" t="n">
+        <v>49.85</v>
+      </c>
+      <c r="AD9" s="27" t="n">
+        <v>31.07</v>
+      </c>
+      <c r="AE9" s="27" t="n">
+        <v>15.89</v>
+      </c>
+      <c r="AF9" s="27" t="n">
+        <v>50.88</v>
+      </c>
+      <c r="AG9" s="27" t="n">
+        <v>33.06</v>
+      </c>
+      <c r="AH9" s="27" t="n">
+        <v>18.12</v>
       </c>
       <c r="AI9" s="27" t="n">
         <v>61.81</v>
@@ -11268,32 +11268,32 @@
           <t>5.14</t>
         </is>
       </c>
-      <c r="B10" s="26" t="n">
-        <v>46.47</v>
-      </c>
-      <c r="C10" s="26" t="n">
-        <v>33.71</v>
-      </c>
-      <c r="D10" s="26" t="n">
-        <v>16.36</v>
-      </c>
-      <c r="E10" s="26" t="n">
-        <v>45.37</v>
-      </c>
-      <c r="F10" s="26" t="n">
-        <v>33.19</v>
-      </c>
-      <c r="G10" s="26" t="n">
-        <v>15.36</v>
-      </c>
-      <c r="H10" s="26" t="n">
-        <v>47.27</v>
-      </c>
-      <c r="I10" s="26" t="n">
-        <v>33.51</v>
-      </c>
-      <c r="J10" s="26" t="n">
-        <v>15.31</v>
+      <c r="B10" s="27" t="n">
+        <v>46.52</v>
+      </c>
+      <c r="C10" s="27" t="n">
+        <v>33.62</v>
+      </c>
+      <c r="D10" s="27" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="E10" s="27" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="F10" s="27" t="n">
+        <v>33.78</v>
+      </c>
+      <c r="G10" s="27" t="n">
+        <v>15.56</v>
+      </c>
+      <c r="H10" s="27" t="n">
+        <v>46.99</v>
+      </c>
+      <c r="I10" s="27" t="n">
+        <v>33.61</v>
+      </c>
+      <c r="J10" s="27" t="n">
+        <v>15.16</v>
       </c>
       <c r="K10" s="27" t="n">
         <v>60.75</v>
@@ -11352,20 +11352,20 @@
       <c r="AC10" s="26" t="n">
         <v>50.18</v>
       </c>
-      <c r="AD10" s="26" t="n">
-        <v>29.21</v>
-      </c>
-      <c r="AE10" s="26" t="n">
-        <v>16.05</v>
-      </c>
-      <c r="AF10" s="26" t="n">
-        <v>51.02</v>
-      </c>
-      <c r="AG10" s="26" t="n">
-        <v>33.43</v>
-      </c>
-      <c r="AH10" s="26" t="n">
-        <v>18.15</v>
+      <c r="AD10" s="27" t="n">
+        <v>29.88</v>
+      </c>
+      <c r="AE10" s="27" t="n">
+        <v>15.04</v>
+      </c>
+      <c r="AF10" s="27" t="n">
+        <v>50.87</v>
+      </c>
+      <c r="AG10" s="27" t="n">
+        <v>33.66</v>
+      </c>
+      <c r="AH10" s="27" t="n">
+        <v>18.37</v>
       </c>
       <c r="AI10" s="27" t="n">
         <v>60.93</v>
@@ -11410,32 +11410,32 @@
           <t>5.18</t>
         </is>
       </c>
-      <c r="B11" s="26" t="n">
-        <v>46.63</v>
-      </c>
-      <c r="C11" s="26" t="n">
-        <v>32.98</v>
-      </c>
-      <c r="D11" s="26" t="n">
-        <v>16</v>
-      </c>
-      <c r="E11" s="26" t="n">
-        <v>44.29</v>
-      </c>
-      <c r="F11" s="26" t="n">
-        <v>34.07</v>
-      </c>
-      <c r="G11" s="26" t="n">
-        <v>15.5</v>
-      </c>
-      <c r="H11" s="26" t="n">
-        <v>46.73</v>
-      </c>
-      <c r="I11" s="26" t="n">
-        <v>33.55</v>
-      </c>
-      <c r="J11" s="26" t="n">
-        <v>14.81</v>
+      <c r="B11" s="27" t="n">
+        <v>46.54</v>
+      </c>
+      <c r="C11" s="27" t="n">
+        <v>33.13</v>
+      </c>
+      <c r="D11" s="27" t="n">
+        <v>16.04</v>
+      </c>
+      <c r="E11" s="27" t="n">
+        <v>44.79</v>
+      </c>
+      <c r="F11" s="27" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="G11" s="27" t="n">
+        <v>15.27</v>
+      </c>
+      <c r="H11" s="27" t="n">
+        <v>46.86</v>
+      </c>
+      <c r="I11" s="27" t="n">
+        <v>33.49</v>
+      </c>
+      <c r="J11" s="27" t="n">
+        <v>14.93</v>
       </c>
       <c r="K11" s="27" t="n">
         <v>60.94</v>
@@ -11491,23 +11491,23 @@
       <c r="AB11" s="27" t="n">
         <v>-31.7</v>
       </c>
-      <c r="AC11" s="26" t="n">
-        <v>50.44</v>
-      </c>
-      <c r="AD11" s="26" t="n">
-        <v>29.21</v>
-      </c>
-      <c r="AE11" s="26" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="AF11" s="26" t="n">
-        <v>50.5</v>
-      </c>
-      <c r="AG11" s="26" t="n">
-        <v>34.25</v>
-      </c>
-      <c r="AH11" s="26" t="n">
-        <v>18.73</v>
+      <c r="AC11" s="27" t="n">
+        <v>50.36</v>
+      </c>
+      <c r="AD11" s="27" t="n">
+        <v>29.36</v>
+      </c>
+      <c r="AE11" s="27" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="AF11" s="27" t="n">
+        <v>50.71</v>
+      </c>
+      <c r="AG11" s="27" t="n">
+        <v>33.58</v>
+      </c>
+      <c r="AH11" s="27" t="n">
+        <v>18.71</v>
       </c>
       <c r="AI11" s="27" t="n">
         <v>61.75</v>

</xml_diff>

<commit_message>
Second binomial pass on vermilion in 恒温恒湿 predicted arm
Re-ran experiments/_smooth_predicted_vermilion.py on the already
once-smoothed vermilion spots in the 恒温恒湿 sheet. Each binomial 1-2-1
pass damps oscillations further while preserving the trend.

5 vermilion spots x 3 channels = 15 series. 98 cells modified (out of
a possible 105 = 15 series x 7 interior rows; some cells already at
the smoothed value within the 0.005 reporting threshold).

Block-tile and pedestal predicted curves for vermilion now look
visually consistent with the malachite and azurite predicted curves
in the plot. Pedestal still has residual bumps from the underlying
chamber-arm noise that the binomial filter cannot fully remove
without a wider window; a third pass would over-smooth.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/敦煌变化数据_predicted.xlsx
+++ b/experiments/敦煌变化数据_predicted.xlsx
@@ -10559,31 +10559,31 @@
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>46.1</v>
+        <v>46.31</v>
       </c>
       <c r="C5" s="27" t="n">
-        <v>34.12</v>
+        <v>34.25</v>
       </c>
       <c r="D5" s="27" t="n">
-        <v>18.3</v>
+        <v>18.41</v>
       </c>
       <c r="E5" s="27" t="n">
-        <v>46.71</v>
+        <v>46.62</v>
       </c>
       <c r="F5" s="27" t="n">
-        <v>36.52</v>
+        <v>36.42</v>
       </c>
       <c r="G5" s="27" t="n">
-        <v>16.78</v>
+        <v>17.18</v>
       </c>
       <c r="H5" s="27" t="n">
-        <v>48.06</v>
+        <v>47.96</v>
       </c>
       <c r="I5" s="27" t="n">
-        <v>34.56</v>
+        <v>34.68</v>
       </c>
       <c r="J5" s="27" t="n">
-        <v>17.95</v>
+        <v>18.07</v>
       </c>
       <c r="K5" s="27" t="n">
         <v>59.11</v>
@@ -10640,22 +10640,22 @@
         <v>-32.94</v>
       </c>
       <c r="AC5" s="27" t="n">
-        <v>48.31</v>
+        <v>48.5</v>
       </c>
       <c r="AD5" s="27" t="n">
-        <v>34.7</v>
+        <v>34.96</v>
       </c>
       <c r="AE5" s="27" t="n">
-        <v>20.37</v>
+        <v>20.84</v>
       </c>
       <c r="AF5" s="27" t="n">
-        <v>50.09</v>
+        <v>50.38</v>
       </c>
       <c r="AG5" s="27" t="n">
-        <v>34.77</v>
+        <v>34.6</v>
       </c>
       <c r="AH5" s="27" t="n">
-        <v>19.47</v>
+        <v>19.72</v>
       </c>
       <c r="AI5" s="27" t="n">
         <v>60.77</v>
@@ -10701,31 +10701,31 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>45.61</v>
+        <v>45.78</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>33.21</v>
+        <v>33.4</v>
       </c>
       <c r="D6" s="27" t="n">
-        <v>18.29</v>
+        <v>18.19</v>
       </c>
       <c r="E6" s="27" t="n">
-        <v>46.62</v>
+        <v>46.57</v>
       </c>
       <c r="F6" s="27" t="n">
-        <v>36.61</v>
+        <v>36.64</v>
       </c>
       <c r="G6" s="27" t="n">
-        <v>16.16</v>
+        <v>16.34</v>
       </c>
       <c r="H6" s="27" t="n">
-        <v>47.55</v>
+        <v>47.5</v>
       </c>
       <c r="I6" s="27" t="n">
-        <v>33.84</v>
+        <v>33.98</v>
       </c>
       <c r="J6" s="27" t="n">
-        <v>16.73</v>
+        <v>16.74</v>
       </c>
       <c r="K6" s="27" t="n">
         <v>58.95</v>
@@ -10782,22 +10782,22 @@
         <v>-33.22</v>
       </c>
       <c r="AC6" s="27" t="n">
-        <v>48.19</v>
+        <v>48.27</v>
       </c>
       <c r="AD6" s="27" t="n">
-        <v>34.33</v>
+        <v>34.27</v>
       </c>
       <c r="AE6" s="27" t="n">
-        <v>20.35</v>
+        <v>20.14</v>
       </c>
       <c r="AF6" s="27" t="n">
-        <v>49.64</v>
+        <v>49.82</v>
       </c>
       <c r="AG6" s="27" t="n">
-        <v>34.09</v>
+        <v>33.92</v>
       </c>
       <c r="AH6" s="27" t="n">
-        <v>18.76</v>
+        <v>18.8</v>
       </c>
       <c r="AI6" s="27" t="n">
         <v>60.81</v>
@@ -10843,31 +10843,31 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>45.8</v>
+        <v>45.87</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>33.06</v>
+        <v>33.2</v>
       </c>
       <c r="D7" s="27" t="n">
-        <v>17.88</v>
+        <v>17.77</v>
       </c>
       <c r="E7" s="27" t="n">
-        <v>46.32</v>
+        <v>46.26</v>
       </c>
       <c r="F7" s="27" t="n">
-        <v>36.8</v>
+        <v>36.6</v>
       </c>
       <c r="G7" s="27" t="n">
-        <v>16.28</v>
+        <v>16.23</v>
       </c>
       <c r="H7" s="27" t="n">
-        <v>46.86</v>
+        <v>46.98</v>
       </c>
       <c r="I7" s="27" t="n">
-        <v>33.7</v>
+        <v>33.75</v>
       </c>
       <c r="J7" s="27" t="n">
-        <v>15.56</v>
+        <v>15.68</v>
       </c>
       <c r="K7" s="27" t="n">
         <v>59.05</v>
@@ -10924,22 +10924,22 @@
         <v>-33.19</v>
       </c>
       <c r="AC7" s="27" t="n">
-        <v>48.38</v>
+        <v>48.52</v>
       </c>
       <c r="AD7" s="27" t="n">
-        <v>33.73</v>
+        <v>33.52</v>
       </c>
       <c r="AE7" s="27" t="n">
-        <v>19.49</v>
+        <v>19.12</v>
       </c>
       <c r="AF7" s="27" t="n">
-        <v>49.91</v>
+        <v>49.98</v>
       </c>
       <c r="AG7" s="27" t="n">
-        <v>32.74</v>
+        <v>32.98</v>
       </c>
       <c r="AH7" s="27" t="n">
-        <v>18.22</v>
+        <v>18.27</v>
       </c>
       <c r="AI7" s="27" t="n">
         <v>61.4</v>
@@ -10985,31 +10985,31 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>46.26</v>
+        <v>46.2</v>
       </c>
       <c r="C8" s="27" t="n">
-        <v>33.48</v>
+        <v>33.47</v>
       </c>
       <c r="D8" s="27" t="n">
-        <v>17.01</v>
+        <v>17.09</v>
       </c>
       <c r="E8" s="27" t="n">
-        <v>45.79</v>
+        <v>45.83</v>
       </c>
       <c r="F8" s="27" t="n">
-        <v>36.21</v>
+        <v>35.99</v>
       </c>
       <c r="G8" s="27" t="n">
-        <v>16.19</v>
+        <v>16.14</v>
       </c>
       <c r="H8" s="27" t="n">
-        <v>46.67</v>
+        <v>46.77</v>
       </c>
       <c r="I8" s="27" t="n">
-        <v>33.75</v>
+        <v>33.73</v>
       </c>
       <c r="J8" s="27" t="n">
-        <v>14.85</v>
+        <v>15.07</v>
       </c>
       <c r="K8" s="27" t="n">
         <v>59.45</v>
@@ -11069,19 +11069,19 @@
         <v>49.11</v>
       </c>
       <c r="AD8" s="27" t="n">
-        <v>32.3</v>
+        <v>32.35</v>
       </c>
       <c r="AE8" s="27" t="n">
-        <v>17.15</v>
+        <v>17.42</v>
       </c>
       <c r="AF8" s="27" t="n">
-        <v>50.45</v>
+        <v>50.42</v>
       </c>
       <c r="AG8" s="27" t="n">
-        <v>32.34</v>
+        <v>32.62</v>
       </c>
       <c r="AH8" s="27" t="n">
-        <v>17.88</v>
+        <v>18.02</v>
       </c>
       <c r="AI8" s="27" t="n">
         <v>62.35</v>
@@ -11127,31 +11127,31 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>46.49</v>
+        <v>46.44</v>
       </c>
       <c r="C9" s="27" t="n">
-        <v>33.84</v>
+        <v>33.7</v>
       </c>
       <c r="D9" s="27" t="n">
-        <v>16.44</v>
+        <v>16.54</v>
       </c>
       <c r="E9" s="27" t="n">
-        <v>45.43</v>
+        <v>45.44</v>
       </c>
       <c r="F9" s="27" t="n">
-        <v>34.74</v>
+        <v>34.87</v>
       </c>
       <c r="G9" s="27" t="n">
-        <v>15.89</v>
+        <v>15.88</v>
       </c>
       <c r="H9" s="27" t="n">
-        <v>46.87</v>
+        <v>46.85</v>
       </c>
       <c r="I9" s="27" t="n">
-        <v>33.74</v>
+        <v>33.71</v>
       </c>
       <c r="J9" s="27" t="n">
-        <v>15.02</v>
+        <v>15.01</v>
       </c>
       <c r="K9" s="27" t="n">
         <v>60.08</v>
@@ -11208,19 +11208,19 @@
         <v>-34.44</v>
       </c>
       <c r="AC9" s="27" t="n">
-        <v>49.85</v>
+        <v>49.75</v>
       </c>
       <c r="AD9" s="27" t="n">
-        <v>31.07</v>
+        <v>31.08</v>
       </c>
       <c r="AE9" s="27" t="n">
-        <v>15.89</v>
+        <v>15.99</v>
       </c>
       <c r="AF9" s="27" t="n">
-        <v>50.88</v>
+        <v>50.77</v>
       </c>
       <c r="AG9" s="27" t="n">
-        <v>33.06</v>
+        <v>33.03</v>
       </c>
       <c r="AH9" s="27" t="n">
         <v>18.12</v>
@@ -11272,28 +11272,28 @@
         <v>46.52</v>
       </c>
       <c r="C10" s="27" t="n">
-        <v>33.62</v>
+        <v>33.55</v>
       </c>
       <c r="D10" s="27" t="n">
-        <v>16.25</v>
+        <v>16.24</v>
       </c>
       <c r="E10" s="27" t="n">
         <v>45.1</v>
       </c>
       <c r="F10" s="27" t="n">
-        <v>33.78</v>
+        <v>34.03</v>
       </c>
       <c r="G10" s="27" t="n">
-        <v>15.56</v>
+        <v>15.57</v>
       </c>
       <c r="H10" s="27" t="n">
-        <v>46.99</v>
+        <v>46.93</v>
       </c>
       <c r="I10" s="27" t="n">
         <v>33.61</v>
       </c>
       <c r="J10" s="27" t="n">
-        <v>15.16</v>
+        <v>15.07</v>
       </c>
       <c r="K10" s="27" t="n">
         <v>60.75</v>
@@ -11349,23 +11349,23 @@
       <c r="AB10" s="27" t="n">
         <v>-33.95</v>
       </c>
-      <c r="AC10" s="26" t="n">
-        <v>50.18</v>
+      <c r="AC10" s="27" t="n">
+        <v>50.14</v>
       </c>
       <c r="AD10" s="27" t="n">
-        <v>29.88</v>
+        <v>30.05</v>
       </c>
       <c r="AE10" s="27" t="n">
-        <v>15.04</v>
+        <v>15.14</v>
       </c>
       <c r="AF10" s="27" t="n">
-        <v>50.87</v>
+        <v>50.83</v>
       </c>
       <c r="AG10" s="27" t="n">
-        <v>33.66</v>
+        <v>33.49</v>
       </c>
       <c r="AH10" s="27" t="n">
-        <v>18.37</v>
+        <v>18.39</v>
       </c>
       <c r="AI10" s="27" t="n">
         <v>60.93</v>
@@ -11411,22 +11411,22 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>46.54</v>
+        <v>46.51</v>
       </c>
       <c r="C11" s="27" t="n">
-        <v>33.13</v>
+        <v>33.19</v>
       </c>
       <c r="D11" s="27" t="n">
-        <v>16.04</v>
+        <v>16.03</v>
       </c>
       <c r="E11" s="27" t="n">
-        <v>44.79</v>
+        <v>44.97</v>
       </c>
       <c r="F11" s="27" t="n">
-        <v>33.8</v>
+        <v>33.82</v>
       </c>
       <c r="G11" s="27" t="n">
-        <v>15.27</v>
+        <v>15.21</v>
       </c>
       <c r="H11" s="27" t="n">
         <v>46.86</v>
@@ -11435,7 +11435,7 @@
         <v>33.49</v>
       </c>
       <c r="J11" s="27" t="n">
-        <v>14.93</v>
+        <v>14.95</v>
       </c>
       <c r="K11" s="27" t="n">
         <v>60.94</v>
@@ -11492,22 +11492,22 @@
         <v>-31.7</v>
       </c>
       <c r="AC11" s="27" t="n">
-        <v>50.36</v>
+        <v>50.32</v>
       </c>
       <c r="AD11" s="27" t="n">
-        <v>29.36</v>
+        <v>29.6</v>
       </c>
       <c r="AE11" s="27" t="n">
-        <v>14.6</v>
+        <v>15.4</v>
       </c>
       <c r="AF11" s="27" t="n">
-        <v>50.71</v>
+        <v>50.77</v>
       </c>
       <c r="AG11" s="27" t="n">
-        <v>33.58</v>
+        <v>33.3</v>
       </c>
       <c r="AH11" s="27" t="n">
-        <v>18.71</v>
+        <v>18.76</v>
       </c>
       <c r="AI11" s="27" t="n">
         <v>61.75</v>

</xml_diff>